<commit_message>
atualizacao das anotacoes com a inclusao do git add
</commit_message>
<xml_diff>
--- a/anotacoes_estudo_git.xlsx
+++ b/anotacoes_estudo_git.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>comandos aprendidos git</t>
   </si>
@@ -71,12 +71,24 @@
   <si>
     <t>navegue até a pasta criada para manipular aquivos dentro da pasta setada</t>
   </si>
+  <si>
+    <t>git add .</t>
+  </si>
+  <si>
+    <t>Para que todos os arquivos da pasta atual sejam monitorados.</t>
+  </si>
+  <si>
+    <t>clear</t>
+  </si>
+  <si>
+    <t>limpa a tela do prompt</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -94,13 +106,40 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -115,18 +154,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -407,60 +455,76 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="84.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="84.42578125" style="4" customWidth="1"/>
     <col min="3" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
atualizacao das anotacoes com a inclusao do git commit e rm
</commit_message>
<xml_diff>
--- a/anotacoes_estudo_git.xlsx
+++ b/anotacoes_estudo_git.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>comandos aprendidos git</t>
   </si>
@@ -83,12 +83,68 @@
   <si>
     <t>limpa a tela do prompt</t>
   </si>
+  <si>
+    <t>git commit -m " mensagem de registro"</t>
+  </si>
+  <si>
+    <t>git rm</t>
+  </si>
+  <si>
+    <t>remover o arquivo e para que o mesmo deixe de ser monitorado</t>
+  </si>
+  <si>
+    <r>
+      <t>Queremos salvar as alterações, e o que poderemos entender como sendo um </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>check point</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t> para indicar que houve mudança, seria o </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>commit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>, que precisa ter modificações, que já adicionamos, mas também precisa ter uma mensagem, o que criaremos agora. Por já termos adicionado as modificações a serem enviadas, executaremos simplesmente </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>git commit -m "Criando arquivo index.html com</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,6 +182,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -154,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -174,6 +242,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -455,10 +526,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="84.42578125" style="4" customWidth="1"/>
     <col min="3" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -527,6 +598,22 @@
         <v>15</v>
       </c>
     </row>
+    <row r="9" spans="1:2" ht="78" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
atualizacao das anotacoes com a inclusao do git log e git log -p
</commit_message>
<xml_diff>
--- a/anotacoes_estudo_git.xlsx
+++ b/anotacoes_estudo_git.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>comandos aprendidos git</t>
   </si>
@@ -137,6 +137,37 @@
         <family val="2"/>
       </rPr>
       <t>git commit -m "Criando arquivo index.html com</t>
+    </r>
+  </si>
+  <si>
+    <t>git log</t>
+  </si>
+  <si>
+    <t>poderemos verificar o histórico de alterações, cada mensagem de commits feitos, o andamento do nosso projeto e outras diversas informações</t>
+  </si>
+  <si>
+    <t>git log -p</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">poderemos verificar o histórico de alterações, cada mensagem de commits feitos, o andamento do nosso projeto e outras diversas informações </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>E MOSTRARÁ TAMBEM A PROPRIA MUDANÇA NA TELA DE COMO ERA PRA COMO FICOU.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
     </r>
   </si>
 </sst>
@@ -526,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.28515625" style="5" bestFit="1" customWidth="1"/>
@@ -614,6 +645,22 @@
         <v>18</v>
       </c>
     </row>
+    <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="44.25" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
atualização na planilha de aanotações git pull
</commit_message>
<xml_diff>
--- a/anotacoes_estudo_git.xlsx
+++ b/anotacoes_estudo_git.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="45">
   <si>
     <t>comandos aprendidos git</t>
   </si>
@@ -56,79 +56,128 @@
     <t>mostra o estado do nosso repositório, ou seja, quais arquivos foram alterados, ou não</t>
   </si>
   <si>
-    <r>
-      <t>git init</t>
-    </r>
-    <r>
-      <rPr>
+    <t>navegue até a pasta criada para manipular aquivos dentro da pasta setada</t>
+  </si>
+  <si>
+    <t>git add .</t>
+  </si>
+  <si>
+    <t>Para que todos os arquivos da pasta atual sejam monitorados.</t>
+  </si>
+  <si>
+    <t>clear</t>
+  </si>
+  <si>
+    <t>limpa a tela do prompt</t>
+  </si>
+  <si>
+    <t>git commit -m " mensagem de registro"</t>
+  </si>
+  <si>
+    <t>git rm</t>
+  </si>
+  <si>
+    <t>remover o arquivo e para que o mesmo deixe de ser monitorado</t>
+  </si>
+  <si>
+    <r>
+      <t>Queremos salvar as alterações, e o que poderemos entender como sendo um </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="11"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t> inicializa um repositório no diretório em que o comando for executado. A partir deste comando, o Git poderá gerenciar as modificações realizadas nos arquivos.</t>
-    </r>
-  </si>
-  <si>
-    <t>navegue até a pasta criada para manipular aquivos dentro da pasta setada</t>
-  </si>
-  <si>
-    <t>git add .</t>
-  </si>
-  <si>
-    <t>Para que todos os arquivos da pasta atual sejam monitorados.</t>
-  </si>
-  <si>
-    <t>clear</t>
-  </si>
-  <si>
-    <t>limpa a tela do prompt</t>
-  </si>
-  <si>
-    <t>git commit -m " mensagem de registro"</t>
-  </si>
-  <si>
-    <t>git rm</t>
-  </si>
-  <si>
-    <t>remover o arquivo e para que o mesmo deixe de ser monitorado</t>
-  </si>
-  <si>
-    <r>
-      <t>Queremos salvar as alterações, e o que poderemos entender como sendo um </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
+      <t>check point</t>
+    </r>
+    <r>
+      <rPr>
         <sz val="11"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>check point</t>
-    </r>
-    <r>
-      <rPr>
+      <t> para indicar que houve mudança, seria o </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
         <sz val="11"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t> para indicar que houve mudança, seria o </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
+      <t>commit</t>
+    </r>
+    <r>
+      <rPr>
         <sz val="11"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>commit</t>
-    </r>
-    <r>
-      <rPr>
+      <t>, que precisa ter modificações, que já adicionamos, mas também precisa ter uma mensagem, o que criaremos agora. Por já termos adicionado as modificações a serem enviadas, executaremos simplesmente </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>git commit -m "Criando arquivo index.html com</t>
+    </r>
+  </si>
+  <si>
+    <t>git log</t>
+  </si>
+  <si>
+    <t>poderemos verificar o histórico de alterações, cada mensagem de commits feitos, o andamento do nosso projeto e outras diversas informações</t>
+  </si>
+  <si>
+    <t>git log -p</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">poderemos verificar o histórico de alterações, cada mensagem de commits feitos, o andamento do nosso projeto e outras diversas informações </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
         <sz val="11"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>, que precisa ter modificações, que já adicionamos, mas também precisa ter uma mensagem, o que criaremos agora. Por já termos adicionado as modificações a serem enviadas, executaremos simplesmente </t>
+      <t>E MOSTRARÁ TAMBEM A PROPRIA MUDANÇA NA TELA DE COMO ERA PRA COMO FICOU.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>cd ..</t>
+  </si>
+  <si>
+    <t>para nos localizarmos na pasta superior</t>
+  </si>
+  <si>
+    <t>mkdir nome_pasta</t>
+  </si>
+  <si>
+    <t>git init -- bare</t>
+  </si>
+  <si>
+    <t>git remote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lista todos os repositorios remotos </t>
+  </si>
+  <si>
+    <r>
+      <t>criaremos a pasta "nome_pasta" por meio do comando </t>
     </r>
     <r>
       <rPr>
@@ -136,38 +185,157 @@
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
       </rPr>
-      <t>git commit -m "Criando arquivo index.html com</t>
-    </r>
-  </si>
-  <si>
-    <t>git log</t>
-  </si>
-  <si>
-    <t>poderemos verificar o histórico de alterações, cada mensagem de commits feitos, o andamento do nosso projeto e outras diversas informações</t>
-  </si>
-  <si>
-    <t>git log -p</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">poderemos verificar o histórico de alterações, cada mensagem de commits feitos, o andamento do nosso projeto e outras diversas informações </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
+      <t>mkdir</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>cria um repositório do Git que somente armazenará as alterações, não o acessaremos para editar arquivos, por exemplo, usaremos </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>git init --bare</t>
+    </r>
+    <r>
+      <rPr>
         <sz val="11"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>E MOSTRARÁ TAMBEM A PROPRIA MUDANÇA NA TELA DE COMO ERA PRA COMO FICOU.</t>
-    </r>
-    <r>
-      <rPr>
+      <t>, cujo parâmetro indica que este repositório é </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
         <sz val="11"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
+      <t>puro</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>, que contém apenas as alterações dos arquivos, e não uma cópia física de cada um dos arquivos.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">git remote add </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nome</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C:/diretorio/diretorio</t>
+    </r>
+  </si>
+  <si>
+    <t>para adicionar um novo repositorio remoto inserindo um nome para o mesmo e  também incluiremos um caminho, que poderá ser uma URL de um servidor pela internet, um endereço na rede, inclusive de outro computador, qualquer endereço válido para um repositório Git</t>
+  </si>
+  <si>
+    <t>git remote -v</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mostra o endereço do servidor criado </t>
+  </si>
+  <si>
+    <t xml:space="preserve">git clone </t>
+  </si>
+  <si>
+    <t>git init inicializa um repositório no diretório em que o comando for executado. A partir deste comando, o Git poderá gerenciar as modificações realizadas nos arquivos.</t>
+  </si>
+  <si>
+    <t>git puch   nome_servidor   master</t>
+  </si>
+  <si>
+    <t>assim, serão enviados todos os dados por todos os códigos e alterações feitas até então para nosso repositório que chamamos de "local", dentro de "servidor".</t>
+  </si>
+  <si>
+    <t>git pull</t>
+  </si>
+  <si>
+    <t>para puxar uma copia do servidor para seu repositorio utiliza esse comando git pull</t>
+  </si>
+  <si>
+    <r>
+      <t>git init</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t> define que aquela pasta será um repositório. A partir deste comando, o Git poderá gerenciar as modificações realizadas nos arquivos.</t>
+    </r>
+  </si>
+  <si>
+    <t>muda o nome do repositorio</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">git remote rename </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nomeatual novonome</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">git pull </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nomerepositorio branch</t>
     </r>
   </si>
 </sst>
@@ -175,7 +343,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,6 +393,28 @@
       <sz val="11"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF3D464D"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -253,7 +443,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -261,7 +451,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -274,8 +463,17 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -557,108 +755,188 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="84.42578125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="39.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84.42578125" style="3" customWidth="1"/>
     <col min="3" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="B7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="B8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="4" t="s">
+    </row>
+    <row r="9" spans="1:2" ht="78" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="78" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="B9" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B10" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="B11" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="8" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="44.25" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="44.25" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
+      <c r="B12" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="8" t="s">
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>23</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="61.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="56.25" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>